<commit_message>
feat: implement core UI components, protocol decoding logic, and telemetry pipeline architecture
</commit_message>
<xml_diff>
--- a/Experiment1_frame_config.xlsx
+++ b/Experiment1_frame_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A15D2DD-E26D-4172-9FBE-99B3C69D165B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8E90F9-91C6-42F5-AC62-9712283B6FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="12160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Protocol" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,12 @@
     <sheet name="PollingSchedule" sheetId="9" r:id="rId9"/>
     <sheet name="SerialDefaults" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="173">
   <si>
     <t>profile_name</t>
   </si>
@@ -124,99 +124,105 @@
     <t>description</t>
   </si>
   <si>
-    <t>0x1001</t>
+    <t>0x1000</t>
+  </si>
+  <si>
+    <t>0x2000</t>
+  </si>
+  <si>
+    <t>0x3000</t>
+  </si>
+  <si>
+    <t>0x4000</t>
+  </si>
+  <si>
+    <t>0x5000</t>
+  </si>
+  <si>
+    <t>0x6000</t>
+  </si>
+  <si>
+    <t>0x6001</t>
+  </si>
+  <si>
+    <t>0x6002</t>
+  </si>
+  <si>
+    <t>0x6003</t>
+  </si>
+  <si>
+    <t>0x6004</t>
+  </si>
+  <si>
+    <t>Cell Data</t>
+  </si>
+  <si>
+    <t>Board Parameters</t>
+  </si>
+  <si>
+    <t>Algorithm Faults</t>
+  </si>
+  <si>
+    <t>Protection Threshold</t>
+  </si>
+  <si>
+    <t>Estimation Values</t>
   </si>
   <si>
     <t>Cell Relay Control</t>
   </si>
   <si>
+    <t>Cell Charge Select</t>
+  </si>
+  <si>
+    <t>Cell Charge Control</t>
+  </si>
+  <si>
+    <t>Cell Discharge Control</t>
+  </si>
+  <si>
+    <t>Cell Discharge Select</t>
+  </si>
+  <si>
+    <t>rx</t>
+  </si>
+  <si>
     <t>rxtx</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Cell Voltages &amp; Temperatures</t>
+  </si>
+  <si>
+    <t>Board Ambient &amp; System Voltages</t>
+  </si>
+  <si>
+    <t>Algorithm Fault Flags</t>
+  </si>
+  <si>
+    <t>Protection Threshold Limits</t>
+  </si>
+  <si>
+    <t>SOC Estimation Values</t>
+  </si>
+  <si>
     <t>Relay control (Cell Enable, Cell Select)</t>
   </si>
   <si>
-    <t>0x1002</t>
-  </si>
-  <si>
-    <t>Cell Charge Select</t>
-  </si>
-  <si>
     <t>Charge parameters (Max Charge Voltage, Current 1 &amp; 2)</t>
   </si>
   <si>
-    <t>0x1003</t>
-  </si>
-  <si>
-    <t>Cell Charge Control</t>
-  </si>
-  <si>
     <t>Charge control (Charge Enable, Charge Comparator Reset)</t>
   </si>
   <si>
-    <t>0x1004</t>
-  </si>
-  <si>
-    <t>Cell Discharge Control</t>
-  </si>
-  <si>
     <t>Discharge control (Discharge Enable, Discharge Comparator Reset)</t>
   </si>
   <si>
-    <t>0x1005</t>
-  </si>
-  <si>
-    <t>Cell Discharge Select</t>
-  </si>
-  <si>
     <t>Discharge load selection (Discharge Load 1..4)</t>
   </si>
   <si>
-    <t>Cell Data</t>
-  </si>
-  <si>
-    <t>rx</t>
-  </si>
-  <si>
-    <t>Cell Voltages &amp; Temperatures</t>
-  </si>
-  <si>
-    <t>0x2000</t>
-  </si>
-  <si>
-    <t>Board Parameters</t>
-  </si>
-  <si>
-    <t>Board Ambient &amp; System Voltages</t>
-  </si>
-  <si>
-    <t>0x3000</t>
-  </si>
-  <si>
-    <t>Algorithm Faults</t>
-  </si>
-  <si>
-    <t>Algorithm Fault Flags</t>
-  </si>
-  <si>
-    <t>0x4000</t>
-  </si>
-  <si>
-    <t>Protection Threshold</t>
-  </si>
-  <si>
-    <t>Protection Threshold Limits</t>
-  </si>
-  <si>
-    <t>0x5000</t>
-  </si>
-  <si>
-    <t>Estimation Values</t>
-  </si>
-  <si>
-    <t>SOC Estimation Values</t>
-  </si>
-  <si>
     <t>id_or_address</t>
   </si>
   <si>
@@ -256,216 +262,216 @@
     <t>CellVoltage</t>
   </si>
   <si>
+    <t>CellCurrent</t>
+  </si>
+  <si>
+    <t>CellTerminalTemperature</t>
+  </si>
+  <si>
+    <t>CellBodyTemperature</t>
+  </si>
+  <si>
+    <t>AmbientTemperature</t>
+  </si>
+  <si>
+    <t>ChargeVoltage</t>
+  </si>
+  <si>
+    <t>LoadVoltage</t>
+  </si>
+  <si>
+    <t>Faults</t>
+  </si>
+  <si>
+    <t>OVc</t>
+  </si>
+  <si>
+    <t>UVc</t>
+  </si>
+  <si>
+    <t>OCc</t>
+  </si>
+  <si>
+    <t>OCdc</t>
+  </si>
+  <si>
+    <t>OTc</t>
+  </si>
+  <si>
+    <t>UTc</t>
+  </si>
+  <si>
+    <t>OCV_SOC</t>
+  </si>
+  <si>
+    <t>CC_SOC</t>
+  </si>
+  <si>
+    <t>Cell Enable</t>
+  </si>
+  <si>
+    <t>Cell Select</t>
+  </si>
+  <si>
+    <t>Max Charge Voltage</t>
+  </si>
+  <si>
+    <t>Max Charge Current 1</t>
+  </si>
+  <si>
+    <t>Max Charge Current 2</t>
+  </si>
+  <si>
+    <t>Charge Enable</t>
+  </si>
+  <si>
+    <t>Charge Comparator Reset</t>
+  </si>
+  <si>
+    <t>Discharge Enable</t>
+  </si>
+  <si>
+    <t>Discharge Comparator Reset</t>
+  </si>
+  <si>
+    <t>Discharge Load 1</t>
+  </si>
+  <si>
+    <t>Discharge Load 2</t>
+  </si>
+  <si>
+    <t>Discharge Load 3</t>
+  </si>
+  <si>
+    <t>Discharge Load 4</t>
+  </si>
+  <si>
     <t>uint16</t>
   </si>
   <si>
+    <t>int16</t>
+  </si>
+  <si>
+    <t>boolean</t>
+  </si>
+  <si>
     <t>V</t>
   </si>
   <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Bitfields</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>Relay</t>
+  </si>
+  <si>
+    <t>Charge</t>
+  </si>
+  <si>
+    <t>Discharge</t>
+  </si>
+  <si>
     <t>R</t>
   </si>
   <si>
+    <t>RW</t>
+  </si>
+  <si>
     <t>Cell Terminal Voltage</t>
   </si>
   <si>
-    <t>CellCurrent</t>
-  </si>
-  <si>
-    <t>int16</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
     <t>Cell Current</t>
   </si>
   <si>
-    <t>CellTerminalTemperature</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>Terminal Temp</t>
   </si>
   <si>
-    <t>CellBodyTemperature</t>
-  </si>
-  <si>
     <t>Surface Temp</t>
   </si>
   <si>
-    <t>AmbientTemperature</t>
-  </si>
-  <si>
     <t>Ambient Temp</t>
   </si>
   <si>
-    <t>ChargeVoltage</t>
-  </si>
-  <si>
     <t>Charger Voltage</t>
   </si>
   <si>
-    <t>LoadVoltage</t>
-  </si>
-  <si>
     <t>Load Voltage</t>
   </si>
   <si>
-    <t>Faults</t>
-  </si>
-  <si>
-    <t>Bitfields</t>
-  </si>
-  <si>
     <t>Fault Flags</t>
   </si>
   <si>
-    <t>OVc</t>
-  </si>
-  <si>
     <t>Over-Voltage Limit</t>
   </si>
   <si>
-    <t>UVc</t>
-  </si>
-  <si>
     <t>Under-Voltage Limit</t>
   </si>
   <si>
-    <t>OCc</t>
-  </si>
-  <si>
     <t>Over-Current Charge Limit</t>
   </si>
   <si>
-    <t>OCdc</t>
-  </si>
-  <si>
     <t>Over-Current Discharge Limit</t>
   </si>
   <si>
-    <t>OTc</t>
-  </si>
-  <si>
     <t>Over-Temp Limit</t>
   </si>
   <si>
-    <t>UTc</t>
-  </si>
-  <si>
     <t>Under-Temp Limit</t>
   </si>
   <si>
-    <t>OCV_SOC</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
     <t>Open-Circuit Voltage SOC</t>
   </si>
   <si>
-    <t>CC_SOC</t>
-  </si>
-  <si>
     <t>Coulomb Counting SOC</t>
   </si>
   <si>
-    <t>Cell Enable</t>
-  </si>
-  <si>
-    <t>boolean</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>Relay</t>
-  </si>
-  <si>
-    <t>RW</t>
-  </si>
-  <si>
     <t>Cell Enable Relay Status</t>
   </si>
   <si>
-    <t>Cell Select</t>
-  </si>
-  <si>
     <t>Cell Select Relay Status</t>
   </si>
   <si>
-    <t>Max Charge Voltage</t>
-  </si>
-  <si>
-    <t>Charge</t>
-  </si>
-  <si>
     <t>Max Charge Voltage Status</t>
   </si>
   <si>
-    <t>Max Charge Current 1</t>
-  </si>
-  <si>
     <t>Max Charge Current 1 Status</t>
   </si>
   <si>
-    <t>Max Charge Current 2</t>
-  </si>
-  <si>
     <t>Max Charge Current 2 Status</t>
   </si>
   <si>
-    <t>Charge Enable</t>
-  </si>
-  <si>
     <t>Charge Enable Status</t>
   </si>
   <si>
-    <t>Charge Comparator Reset</t>
-  </si>
-  <si>
     <t>Charge Comparator Reset Status</t>
   </si>
   <si>
-    <t>Discharge Enable</t>
-  </si>
-  <si>
-    <t>Discharge</t>
-  </si>
-  <si>
     <t>Discharge Enable Status</t>
   </si>
   <si>
-    <t>Discharge Comparator Reset</t>
-  </si>
-  <si>
     <t>Discharge Comparator Reset Status</t>
   </si>
   <si>
-    <t>Discharge Load 1</t>
-  </si>
-  <si>
     <t>Discharge Load 1 Status</t>
   </si>
   <si>
-    <t>Discharge Load 2</t>
-  </si>
-  <si>
     <t>Discharge Load 2 Status</t>
   </si>
   <si>
-    <t>Discharge Load 3</t>
-  </si>
-  <si>
     <t>Discharge Load 3 Status</t>
   </si>
   <si>
-    <t>Discharge Load 4</t>
-  </si>
-  <si>
     <t>Discharge Load 4 Status</t>
   </si>
   <si>
@@ -484,27 +490,27 @@
     <t>Overvoltage Fault</t>
   </si>
   <si>
+    <t>Undervoltage Fault</t>
+  </si>
+  <si>
+    <t>Overcurrent Charge Fault</t>
+  </si>
+  <si>
+    <t>Overcurrent Discharge Fault</t>
+  </si>
+  <si>
+    <t>Overtemperature Fault</t>
+  </si>
+  <si>
+    <t>Undertemperature Fault</t>
+  </si>
+  <si>
     <t>FAULT</t>
   </si>
   <si>
     <t>OK</t>
   </si>
   <si>
-    <t>Undervoltage Fault</t>
-  </si>
-  <si>
-    <t>Overcurrent Charge Fault</t>
-  </si>
-  <si>
-    <t>Overcurrent Discharge Fault</t>
-  </si>
-  <si>
-    <t>Overtemperature Fault</t>
-  </si>
-  <si>
-    <t>Undertemperature Fault</t>
-  </si>
-  <si>
     <t>value</t>
   </si>
   <si>
@@ -542,34 +548,13 @@
   </si>
   <si>
     <t>N</t>
-  </si>
-  <si>
-    <t>0x1000</t>
-  </si>
-  <si>
-    <t>0x6000</t>
-  </si>
-  <si>
-    <t>0x6001</t>
-  </si>
-  <si>
-    <t>0x6002</t>
-  </si>
-  <si>
-    <t>0x6003</t>
-  </si>
-  <si>
-    <t>0x6004</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -580,10 +565,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="8"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -647,9 +629,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -687,7 +669,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -721,6 +703,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -755,9 +738,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1041,7 +1025,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1052,19 +1036,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -1078,26 +1062,21 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E2">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="57.90625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1121,212 +1100,211 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C2">
         <v>8</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E2" t="b">
+        <v>51</v>
+      </c>
+      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C3">
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" t="b">
+        <v>51</v>
+      </c>
+      <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="C4">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" t="b">
+        <v>51</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C5">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E5" t="b">
+        <v>51</v>
+      </c>
+      <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="C6">
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" t="b">
+        <v>51</v>
+      </c>
+      <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>172</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" t="b">
+        <v>52</v>
+      </c>
+      <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>173</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="b">
+        <v>52</v>
+      </c>
+      <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>174</v>
+        <v>38</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" t="b">
+        <v>52</v>
+      </c>
+      <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" t="b">
+        <v>52</v>
+      </c>
+      <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>176</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E11" t="b">
+        <v>52</v>
+      </c>
+      <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D33" t="s">
-        <v>177</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D12" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1334,43 +1312,57 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="27.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>30</v>
@@ -1381,13 +1373,13 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1402,16 +1394,16 @@
         <v>0</v>
       </c>
       <c r="H2" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J2" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
+        <v>119</v>
       </c>
       <c r="N2" t="b">
         <v>1</v>
@@ -1419,13 +1411,13 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1440,16 +1432,16 @@
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="I3" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J3" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M3" t="s">
-        <v>82</v>
+        <v>120</v>
       </c>
       <c r="N3" t="b">
         <v>1</v>
@@ -1457,13 +1449,13 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1478,16 +1470,16 @@
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="I4" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J4" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M4" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="N4" t="b">
         <v>1</v>
@@ -1495,13 +1487,13 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1516,16 +1508,16 @@
         <v>0</v>
       </c>
       <c r="H5" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="J5" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M5" t="s">
-        <v>87</v>
+        <v>122</v>
       </c>
       <c r="N5" t="b">
         <v>1</v>
@@ -1533,13 +1525,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1554,16 +1546,16 @@
         <v>0</v>
       </c>
       <c r="H6" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="I6" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J6" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M6" t="s">
-        <v>89</v>
+        <v>123</v>
       </c>
       <c r="N6" t="b">
         <v>1</v>
@@ -1571,13 +1563,13 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1592,16 +1584,16 @@
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J7" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M7" t="s">
-        <v>91</v>
+        <v>124</v>
       </c>
       <c r="N7" t="b">
         <v>1</v>
@@ -1609,13 +1601,13 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1630,16 +1622,16 @@
         <v>0</v>
       </c>
       <c r="H8" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="J8" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M8" t="s">
-        <v>93</v>
+        <v>125</v>
       </c>
       <c r="N8" t="b">
         <v>1</v>
@@ -1647,13 +1639,13 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1668,16 +1660,16 @@
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J9" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M9" t="s">
-        <v>96</v>
+        <v>126</v>
       </c>
       <c r="N9" t="b">
         <v>1</v>
@@ -1685,13 +1677,13 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -1706,16 +1698,16 @@
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I10" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J10" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M10" t="s">
-        <v>98</v>
+        <v>127</v>
       </c>
       <c r="N10" t="b">
         <v>1</v>
@@ -1723,13 +1715,13 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D11">
         <v>1</v>
@@ -1744,16 +1736,16 @@
         <v>0</v>
       </c>
       <c r="H11" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="I11" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J11" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M11" t="s">
-        <v>100</v>
+        <v>128</v>
       </c>
       <c r="N11" t="b">
         <v>1</v>
@@ -1761,13 +1753,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>86</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1782,16 +1774,16 @@
         <v>0</v>
       </c>
       <c r="H12" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="I12" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J12" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M12" t="s">
-        <v>102</v>
+        <v>129</v>
       </c>
       <c r="N12" t="b">
         <v>1</v>
@@ -1799,13 +1791,13 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B13" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1820,16 +1812,16 @@
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="I13" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J13" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M13" t="s">
-        <v>104</v>
+        <v>130</v>
       </c>
       <c r="N13" t="b">
         <v>1</v>
@@ -1837,13 +1829,13 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" t="s">
         <v>105</v>
-      </c>
-      <c r="C14" t="s">
-        <v>75</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1858,16 +1850,16 @@
         <v>0</v>
       </c>
       <c r="H14" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="I14" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J14" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M14" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="N14" t="b">
         <v>1</v>
@@ -1875,13 +1867,13 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1896,16 +1888,16 @@
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="I15" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="J15" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M15" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="N15" t="b">
         <v>1</v>
@@ -1913,13 +1905,13 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1934,16 +1926,16 @@
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I16" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="J16" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M16" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="N16" t="b">
         <v>1</v>
@@ -1951,13 +1943,13 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>91</v>
       </c>
       <c r="C17" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="D17">
         <v>1</v>
@@ -1972,16 +1964,16 @@
         <v>0</v>
       </c>
       <c r="H17" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="I17" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="J17" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="M17" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="N17" t="b">
         <v>1</v>
@@ -1989,31 +1981,31 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B18" t="s">
+        <v>92</v>
+      </c>
+      <c r="C18" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>22</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>113</v>
+      </c>
+      <c r="I18" t="s">
         <v>114</v>
-      </c>
-      <c r="C18" t="s">
-        <v>115</v>
-      </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
-      <c r="E18" t="s">
-        <v>22</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18" t="s">
-        <v>116</v>
-      </c>
-      <c r="I18" t="s">
-        <v>117</v>
       </c>
       <c r="J18" t="s">
         <v>118</v>
@@ -2025,7 +2017,7 @@
         <v>1</v>
       </c>
       <c r="M18" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="N18" t="b">
         <v>1</v>
@@ -2033,13 +2025,13 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B19" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="C19" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D19">
         <v>1</v>
@@ -2054,10 +2046,10 @@
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="I19" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J19" t="s">
         <v>118</v>
@@ -2069,7 +2061,7 @@
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="N19" t="b">
         <v>1</v>
@@ -2077,31 +2069,31 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B20" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="C20" t="s">
+        <v>107</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>113</v>
+      </c>
+      <c r="I20" t="s">
         <v>115</v>
-      </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
-        <v>22</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20" t="s">
-        <v>116</v>
-      </c>
-      <c r="I20" t="s">
-        <v>123</v>
       </c>
       <c r="J20" t="s">
         <v>118</v>
@@ -2113,7 +2105,7 @@
         <v>1</v>
       </c>
       <c r="M20" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="N20" t="b">
         <v>1</v>
@@ -2121,31 +2113,31 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B21" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="C21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
+        <v>22</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>113</v>
+      </c>
+      <c r="I21" t="s">
         <v>115</v>
-      </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
-        <v>22</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21" t="s">
-        <v>116</v>
-      </c>
-      <c r="I21" t="s">
-        <v>123</v>
       </c>
       <c r="J21" t="s">
         <v>118</v>
@@ -2157,7 +2149,7 @@
         <v>1</v>
       </c>
       <c r="M21" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="N21" t="b">
         <v>1</v>
@@ -2165,31 +2157,31 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>22</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
+        <v>113</v>
+      </c>
+      <c r="I22" t="s">
         <v>115</v>
-      </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22" t="s">
-        <v>22</v>
-      </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22">
-        <v>0</v>
-      </c>
-      <c r="H22" t="s">
-        <v>116</v>
-      </c>
-      <c r="I22" t="s">
-        <v>123</v>
       </c>
       <c r="J22" t="s">
         <v>118</v>
@@ -2201,7 +2193,7 @@
         <v>1</v>
       </c>
       <c r="M22" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="N22" t="b">
         <v>1</v>
@@ -2212,28 +2204,28 @@
         <v>38</v>
       </c>
       <c r="B23" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="C23" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>113</v>
+      </c>
+      <c r="I23" t="s">
         <v>115</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>22</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23" t="s">
-        <v>116</v>
-      </c>
-      <c r="I23" t="s">
-        <v>123</v>
       </c>
       <c r="J23" t="s">
         <v>118</v>
@@ -2245,7 +2237,7 @@
         <v>1</v>
       </c>
       <c r="M23" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="N23" t="b">
         <v>1</v>
@@ -2256,28 +2248,28 @@
         <v>38</v>
       </c>
       <c r="B24" t="s">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="C24" t="s">
+        <v>107</v>
+      </c>
+      <c r="D24">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
+        <v>113</v>
+      </c>
+      <c r="I24" t="s">
         <v>115</v>
-      </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
-        <v>22</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24">
-        <v>0</v>
-      </c>
-      <c r="H24" t="s">
-        <v>116</v>
-      </c>
-      <c r="I24" t="s">
-        <v>123</v>
       </c>
       <c r="J24" t="s">
         <v>118</v>
@@ -2289,7 +2281,7 @@
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="N24" t="b">
         <v>1</v>
@@ -2297,13 +2289,13 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="C25" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D25">
         <v>1</v>
@@ -2318,10 +2310,10 @@
         <v>0</v>
       </c>
       <c r="H25" t="s">
+        <v>113</v>
+      </c>
+      <c r="I25" t="s">
         <v>116</v>
-      </c>
-      <c r="I25" t="s">
-        <v>134</v>
       </c>
       <c r="J25" t="s">
         <v>118</v>
@@ -2333,7 +2325,7 @@
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="N25" t="b">
         <v>1</v>
@@ -2341,13 +2333,13 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>136</v>
+        <v>100</v>
       </c>
       <c r="C26" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D26">
         <v>1</v>
@@ -2362,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H26" t="s">
+        <v>113</v>
+      </c>
+      <c r="I26" t="s">
         <v>116</v>
-      </c>
-      <c r="I26" t="s">
-        <v>134</v>
       </c>
       <c r="J26" t="s">
         <v>118</v>
@@ -2377,7 +2369,7 @@
         <v>1</v>
       </c>
       <c r="M26" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="N26" t="b">
         <v>1</v>
@@ -2385,13 +2377,13 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B27" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D27">
         <v>1</v>
@@ -2406,10 +2398,10 @@
         <v>0</v>
       </c>
       <c r="H27" t="s">
+        <v>113</v>
+      </c>
+      <c r="I27" t="s">
         <v>116</v>
-      </c>
-      <c r="I27" t="s">
-        <v>134</v>
       </c>
       <c r="J27" t="s">
         <v>118</v>
@@ -2421,7 +2413,7 @@
         <v>1</v>
       </c>
       <c r="M27" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="N27" t="b">
         <v>1</v>
@@ -2429,13 +2421,13 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B28" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="C28" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D28">
         <v>1</v>
@@ -2450,10 +2442,10 @@
         <v>0</v>
       </c>
       <c r="H28" t="s">
+        <v>113</v>
+      </c>
+      <c r="I28" t="s">
         <v>116</v>
-      </c>
-      <c r="I28" t="s">
-        <v>134</v>
       </c>
       <c r="J28" t="s">
         <v>118</v>
@@ -2465,7 +2457,7 @@
         <v>1</v>
       </c>
       <c r="M28" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="N28" t="b">
         <v>1</v>
@@ -2473,13 +2465,13 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B29" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D29">
         <v>1</v>
@@ -2494,10 +2486,10 @@
         <v>0</v>
       </c>
       <c r="H29" t="s">
+        <v>113</v>
+      </c>
+      <c r="I29" t="s">
         <v>116</v>
-      </c>
-      <c r="I29" t="s">
-        <v>134</v>
       </c>
       <c r="J29" t="s">
         <v>118</v>
@@ -2509,7 +2501,7 @@
         <v>1</v>
       </c>
       <c r="M29" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N29" t="b">
         <v>1</v>
@@ -2517,13 +2509,13 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D30">
         <v>1</v>
@@ -2538,10 +2530,10 @@
         <v>0</v>
       </c>
       <c r="H30" t="s">
+        <v>113</v>
+      </c>
+      <c r="I30" t="s">
         <v>116</v>
-      </c>
-      <c r="I30" t="s">
-        <v>134</v>
       </c>
       <c r="J30" t="s">
         <v>118</v>
@@ -2553,14 +2545,14 @@
         <v>1</v>
       </c>
       <c r="M30" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="N30" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2571,50 +2563,50 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="E2" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F2" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -2623,18 +2615,18 @@
         <v>153</v>
       </c>
       <c r="E3" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F3" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -2643,18 +2635,18 @@
         <v>154</v>
       </c>
       <c r="E4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C5">
         <v>3</v>
@@ -2663,18 +2655,18 @@
         <v>155</v>
       </c>
       <c r="E5" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F5" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -2683,18 +2675,18 @@
         <v>156</v>
       </c>
       <c r="E6" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F6" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2703,14 +2695,14 @@
         <v>157</v>
       </c>
       <c r="E7" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F7" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2721,20 +2713,20 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2745,13 +2737,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>26</v>
@@ -2761,7 +2753,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2769,23 +2761,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="57.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.90625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>30</v>
@@ -2796,13 +2781,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>172</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -2810,13 +2795,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -2824,13 +2809,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>174</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -2838,13 +2823,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -2852,20 +2837,20 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2876,45 +2861,45 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
@@ -2926,7 +2911,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -2940,13 +2925,13 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -2958,7 +2943,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -2972,13 +2957,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -2990,7 +2975,7 @@
         <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -3004,13 +2989,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>95</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -3022,7 +3007,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -3036,13 +3021,13 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -3054,7 +3039,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -3068,13 +3053,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>97</v>
       </c>
       <c r="C7" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D7" t="s">
         <v>22</v>
@@ -3086,7 +3071,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -3100,13 +3085,13 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>131</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -3118,7 +3103,7 @@
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -3132,13 +3117,13 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
         <v>22</v>
@@ -3150,7 +3135,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -3164,13 +3149,13 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>100</v>
       </c>
       <c r="C10" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
         <v>22</v>
@@ -3182,7 +3167,7 @@
         <v>0</v>
       </c>
       <c r="G10" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -3196,13 +3181,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>138</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
         <v>22</v>
@@ -3214,7 +3199,7 @@
         <v>0</v>
       </c>
       <c r="G11" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H11">
         <v>0</v>
@@ -3228,13 +3213,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
         <v>22</v>
@@ -3246,7 +3231,7 @@
         <v>0</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -3260,13 +3245,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="C13" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
         <v>22</v>
@@ -3278,7 +3263,7 @@
         <v>0</v>
       </c>
       <c r="G13" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -3292,13 +3277,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>144</v>
+        <v>104</v>
       </c>
       <c r="C14" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
@@ -3310,7 +3295,7 @@
         <v>0</v>
       </c>
       <c r="G14" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -3323,7 +3308,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -3334,19 +3319,19 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement high-performance frame decoding engine and UI dashboard architecture
</commit_message>
<xml_diff>
--- a/Experiment1_frame_config.xlsx
+++ b/Experiment1_frame_config.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A8E90F9-91C6-42F5-AC62-9712283B6FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Protocol" sheetId="1" r:id="rId1"/>
@@ -24,7 +18,7 @@
     <sheet name="PollingSchedule" sheetId="9" r:id="rId9"/>
     <sheet name="SerialDefaults" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -553,8 +547,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -617,21 +611,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -669,7 +655,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -703,7 +689,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -738,10 +723,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -914,11 +898,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -977,7 +961,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1015,7 +999,7 @@
         <v>10</v>
       </c>
       <c r="Q2">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="R2">
         <v>1</v>
@@ -1030,11 +1014,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
@@ -1051,7 +1035,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>115200</v>
       </c>
@@ -1074,11 +1058,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1098,7 +1082,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1118,7 +1102,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1138,7 +1122,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1158,7 +1142,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1178,7 +1162,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -1198,7 +1182,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1218,7 +1202,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1238,7 +1222,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1258,7 +1242,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1278,7 +1262,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1298,7 +1282,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6">
       <c r="D12" t="s">
         <v>53</v>
       </c>
@@ -1309,25 +1293,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N30"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.1796875" customWidth="1"/>
-    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="30.90625" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -1371,7 +1341,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1388,7 +1358,7 @@
         <v>22</v>
       </c>
       <c r="F2">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1409,7 +1379,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1426,7 +1396,7 @@
         <v>22</v>
       </c>
       <c r="F3">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1447,7 +1417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -1464,7 +1434,7 @@
         <v>22</v>
       </c>
       <c r="F4">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1485,7 +1455,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1502,7 +1472,7 @@
         <v>22</v>
       </c>
       <c r="F5">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1523,7 +1493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1540,7 +1510,7 @@
         <v>22</v>
       </c>
       <c r="F6">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1561,7 +1531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1578,7 +1548,7 @@
         <v>22</v>
       </c>
       <c r="F7">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1599,7 +1569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1616,7 +1586,7 @@
         <v>22</v>
       </c>
       <c r="F8">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1637,7 +1607,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1675,7 +1645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1692,7 +1662,7 @@
         <v>22</v>
       </c>
       <c r="F10">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1713,7 +1683,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1730,7 +1700,7 @@
         <v>22</v>
       </c>
       <c r="F11">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1751,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1768,7 +1738,7 @@
         <v>22</v>
       </c>
       <c r="F12">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1789,7 +1759,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1806,7 +1776,7 @@
         <v>22</v>
       </c>
       <c r="F13">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1827,7 +1797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -1844,7 +1814,7 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1865,7 +1835,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -1882,7 +1852,7 @@
         <v>22</v>
       </c>
       <c r="F15">
-        <v>1E-3</v>
+        <v>0.001</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1903,7 +1873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -1941,7 +1911,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1979,7 +1949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -2023,7 +1993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -2067,7 +2037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -2111,7 +2081,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -2155,7 +2125,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -2199,7 +2169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -2243,7 +2213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -2287,7 +2257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -2331,7 +2301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -2375,7 +2345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -2419,7 +2389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2463,7 +2433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -2507,7 +2477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -2557,11 +2527,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -2581,7 +2551,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -2601,7 +2571,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -2621,7 +2591,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -2641,7 +2611,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2661,7 +2631,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -2681,7 +2651,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2707,11 +2677,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -2731,11 +2701,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>161</v>
       </c>
@@ -2758,11 +2728,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -2779,7 +2749,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -2793,7 +2763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>47</v>
       </c>
@@ -2807,7 +2777,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -2821,7 +2791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -2835,7 +2805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -2855,11 +2825,11 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -2891,7 +2861,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -2923,7 +2893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -2955,7 +2925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -2987,7 +2957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -3019,7 +2989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -3051,7 +3021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -3083,7 +3053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -3115,7 +3085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -3147,7 +3117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -3179,7 +3149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" t="s">
         <v>50</v>
       </c>
@@ -3211,7 +3181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -3243,7 +3213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -3275,7 +3245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -3313,11 +3283,11 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
feat: implement comprehensive UI framework including main window, diagnostic tools, telemetry pipelines, and dynamic plot orchestration.
</commit_message>
<xml_diff>
--- a/Experiment1_frame_config.xlsx
+++ b/Experiment1_frame_config.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C26827C-0F77-43A4-8FB3-6E1830A289A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Protocol" sheetId="1" r:id="rId1"/>
@@ -18,7 +24,7 @@
     <sheet name="PollingSchedule" sheetId="9" r:id="rId9"/>
     <sheet name="SerialDefaults" sheetId="10" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -547,8 +553,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -611,13 +617,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -655,7 +669,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -689,6 +703,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -723,9 +738,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -898,11 +914,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:19">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -961,7 +977,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:19">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
@@ -1014,11 +1030,11 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>168</v>
       </c>
@@ -1035,7 +1051,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>115200</v>
       </c>
@@ -1058,11 +1074,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -1082,7 +1098,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1102,7 +1118,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>32</v>
       </c>
@@ -1122,7 +1138,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -1142,7 +1158,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1162,7 +1178,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -1182,7 +1198,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -1202,7 +1218,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1222,7 +1238,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -1242,7 +1258,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>39</v>
       </c>
@@ -1262,7 +1278,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>40</v>
       </c>
@@ -1282,7 +1298,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="D12" t="s">
         <v>53</v>
       </c>
@@ -1293,11 +1309,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -1341,7 +1366,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>31</v>
       </c>
@@ -1358,7 +1383,7 @@
         <v>22</v>
       </c>
       <c r="F2">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1372,6 +1397,12 @@
       <c r="J2" t="s">
         <v>117</v>
       </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>5</v>
+      </c>
       <c r="M2" t="s">
         <v>119</v>
       </c>
@@ -1379,7 +1410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -1396,7 +1427,7 @@
         <v>22</v>
       </c>
       <c r="F3">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1410,6 +1441,12 @@
       <c r="J3" t="s">
         <v>117</v>
       </c>
+      <c r="K3">
+        <v>-5</v>
+      </c>
+      <c r="L3">
+        <v>5</v>
+      </c>
       <c r="M3" t="s">
         <v>120</v>
       </c>
@@ -1417,7 +1454,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>31</v>
       </c>
@@ -1434,7 +1471,7 @@
         <v>22</v>
       </c>
       <c r="F4">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1455,7 +1492,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -1472,7 +1509,7 @@
         <v>22</v>
       </c>
       <c r="F5">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1493,7 +1530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -1510,7 +1547,7 @@
         <v>22</v>
       </c>
       <c r="F6">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1531,7 +1568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1548,7 +1585,7 @@
         <v>22</v>
       </c>
       <c r="F7">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1562,6 +1599,12 @@
       <c r="J7" t="s">
         <v>117</v>
       </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>5</v>
+      </c>
       <c r="M7" t="s">
         <v>124</v>
       </c>
@@ -1569,7 +1612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1586,7 +1629,7 @@
         <v>22</v>
       </c>
       <c r="F8">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1600,6 +1643,12 @@
       <c r="J8" t="s">
         <v>117</v>
       </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>5</v>
+      </c>
       <c r="M8" t="s">
         <v>125</v>
       </c>
@@ -1607,7 +1656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1645,7 +1694,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>34</v>
       </c>
@@ -1662,7 +1711,7 @@
         <v>22</v>
       </c>
       <c r="F10">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1676,6 +1725,12 @@
       <c r="J10" t="s">
         <v>117</v>
       </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
+        <v>5</v>
+      </c>
       <c r="M10" t="s">
         <v>127</v>
       </c>
@@ -1683,7 +1738,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>34</v>
       </c>
@@ -1700,7 +1755,7 @@
         <v>22</v>
       </c>
       <c r="F11">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1714,6 +1769,12 @@
       <c r="J11" t="s">
         <v>117</v>
       </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>5</v>
+      </c>
       <c r="M11" t="s">
         <v>128</v>
       </c>
@@ -1721,7 +1782,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>34</v>
       </c>
@@ -1738,7 +1799,7 @@
         <v>22</v>
       </c>
       <c r="F12">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1752,6 +1813,12 @@
       <c r="J12" t="s">
         <v>117</v>
       </c>
+      <c r="K12">
+        <v>-5</v>
+      </c>
+      <c r="L12">
+        <v>5</v>
+      </c>
       <c r="M12" t="s">
         <v>129</v>
       </c>
@@ -1759,7 +1826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>34</v>
       </c>
@@ -1776,7 +1843,7 @@
         <v>22</v>
       </c>
       <c r="F13">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1790,6 +1857,12 @@
       <c r="J13" t="s">
         <v>117</v>
       </c>
+      <c r="K13">
+        <v>-5</v>
+      </c>
+      <c r="L13">
+        <v>5</v>
+      </c>
       <c r="M13" t="s">
         <v>130</v>
       </c>
@@ -1797,7 +1870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>34</v>
       </c>
@@ -1814,7 +1887,7 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1835,7 +1908,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>34</v>
       </c>
@@ -1852,7 +1925,7 @@
         <v>22</v>
       </c>
       <c r="F15">
-        <v>0.001</v>
+        <v>1E-3</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1873,7 +1946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -1904,6 +1977,12 @@
       <c r="J16" t="s">
         <v>117</v>
       </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>100</v>
+      </c>
       <c r="M16" t="s">
         <v>133</v>
       </c>
@@ -1911,7 +1990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1942,6 +2021,12 @@
       <c r="J17" t="s">
         <v>117</v>
       </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>100</v>
+      </c>
       <c r="M17" t="s">
         <v>134</v>
       </c>
@@ -1949,7 +2034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -1993,7 +2078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -2037,7 +2122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -2081,7 +2166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -2125,7 +2210,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -2169,7 +2254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -2213,7 +2298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -2257,7 +2342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -2301,7 +2386,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>39</v>
       </c>
@@ -2345,7 +2430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>40</v>
       </c>
@@ -2389,7 +2474,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>40</v>
       </c>
@@ -2433,7 +2518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>40</v>
       </c>
@@ -2477,7 +2562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -2527,11 +2612,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -2551,7 +2644,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -2571,7 +2664,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -2591,7 +2684,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -2611,7 +2704,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -2631,7 +2724,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -2651,7 +2744,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -2677,11 +2770,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>
@@ -2701,11 +2794,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>161</v>
       </c>
@@ -2728,11 +2821,18 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -2749,7 +2849,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -2763,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>47</v>
       </c>
@@ -2777,7 +2877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>48</v>
       </c>
@@ -2791,7 +2891,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>49</v>
       </c>
@@ -2805,7 +2905,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
@@ -2825,11 +2925,20 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>163</v>
       </c>
@@ -2861,7 +2970,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -2893,7 +3002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -2925,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -2957,7 +3066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -2989,7 +3098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>47</v>
       </c>
@@ -3021,7 +3130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>48</v>
       </c>
@@ -3053,7 +3162,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>48</v>
       </c>
@@ -3085,7 +3194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>49</v>
       </c>
@@ -3117,7 +3226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -3149,7 +3258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>50</v>
       </c>
@@ -3181,7 +3290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>50</v>
       </c>
@@ -3213,7 +3322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -3245,7 +3354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>50</v>
       </c>
@@ -3283,11 +3392,11 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
feat: add analysis suite UI and update tx_pad_length documentation
</commit_message>
<xml_diff>
--- a/Experiment1_frame_config.xlsx
+++ b/Experiment1_frame_config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C26827C-0F77-43A4-8FB3-6E1830A289A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2581320-EB76-41C9-BA31-2C24394CB94E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Protocol" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="471" uniqueCount="174">
   <si>
     <t>profile_name</t>
   </si>
@@ -548,13 +548,16 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>uint8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -566,6 +569,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -917,6 +926,26 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1077,6 +1106,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="57.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
@@ -1146,7 +1183,7 @@
         <v>43</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
         <v>51</v>
@@ -1310,16 +1347,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.90625" customWidth="1"/>
+    <col min="2" max="2" width="25.1796875" customWidth="1"/>
+    <col min="3" max="3" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.7265625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1796875" customWidth="1"/>
     <col min="11" max="11" width="9.81640625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="30.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.90625" customWidth="1"/>
+    <col min="14" max="14" width="7.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
@@ -1664,7 +1708,7 @@
         <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>105</v>
+        <v>173</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -1711,7 +1755,7 @@
         <v>22</v>
       </c>
       <c r="F10">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1755,7 +1799,7 @@
         <v>22</v>
       </c>
       <c r="F11">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1790,7 +1834,7 @@
         <v>86</v>
       </c>
       <c r="C12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D12">
         <v>1</v>
@@ -1799,7 +1843,7 @@
         <v>22</v>
       </c>
       <c r="F12">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G12">
         <v>0</v>
@@ -1834,7 +1878,7 @@
         <v>87</v>
       </c>
       <c r="C13" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1843,7 +1887,7 @@
         <v>22</v>
       </c>
       <c r="F13">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1878,7 +1922,7 @@
         <v>88</v>
       </c>
       <c r="C14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1887,7 +1931,7 @@
         <v>22</v>
       </c>
       <c r="F14">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1916,7 +1960,7 @@
         <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D15">
         <v>1</v>
@@ -1925,7 +1969,7 @@
         <v>22</v>
       </c>
       <c r="F15">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -2606,7 +2650,13 @@
         <v>1</v>
       </c>
     </row>
+    <row r="33" spans="4:4" x14ac:dyDescent="0.35">
+      <c r="D33" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>